<commit_message>
Launch-Auswertung: Checkout-Block (ThriveCart) + Cloud-Schreibpipeline
- CHECKOUT-Abschnitt in launch-auswertung-gelaende.xlsx (Aufrufe/Bestellungen/Conversion),
  Aug-2026-Daten aus ThriveCart product-44 (37 Aufrufe, 7 Bestellungen, 18,9%).
- launch-auswertung-webapp.gs: Apps-Script-Webapp, schreibt Launch-Spalten in die
  Google-Tabelle "Launch-Auswertung Gelaende-Webinar" (Cloud-Master), kopiert Formeln
  bei neuen Spalten mit, laesst Formel-/Notizzeilen unangetastet.
- launch-auswertung-push.ps1: POST an die Webapp (UTF-8-Bytes), Launch je Spalte.
- launch-werte-aug-2026.json: Werte-Vorlage + Testdatensatz.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/webinar-gelaende/launch-auswertung-gelaende.xlsx
+++ b/outputs/webinar-gelaende/launch-auswertung-gelaende.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="121">
   <si>
     <t>Launch-Auswertung Gelände-Webinar</t>
   </si>
@@ -243,6 +243,21 @@
   </si>
   <si>
     <t>22.08.2026 (1 Tag vor Webinar)</t>
+  </si>
+  <si>
+    <t>CHECKOUT (ThriveCart) — Gelände-Programm</t>
+  </si>
+  <si>
+    <t>Checkout-Aufrufe (Bezahlseite)</t>
+  </si>
+  <si>
+    <t>Bestellungen über Checkout</t>
+  </si>
+  <si>
+    <t>Checkout-Conversion (Bestellungen/Aufrufe)</t>
+  </si>
+  <si>
+    <t>Checkout = wie oft die ThriveCart-Bezahlseite (Produkt 44 Gelände-Programm) geöffnet wurde. Aug-2026-Launch, Verkaufsphase 23.–27.08.: 37 Aufrufe → 7 Bestellungen = 18,9 %. Zählt ALLE Besucher der Bezahlseite. Die 7 decken sich exakt mit den 7 Programm-Käufen (Cross-Check). Niedrige Conversion trotz vieler Aufrufe = an der Bezahlseite optimieren (Preis-Darstellung, Teilzahlung sichtbar machen, Vertrauens-Elemente, Ladezeit).</t>
   </si>
   <si>
     <t>Legende: Weiße Felder = du trägst ein. Beige Felder = rechnen sich automatisch. ★ Ad-ROAS = die wichtigste Ads-Kennzahl.</t>
@@ -370,7 +385,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -386,7 +401,7 @@
     <font>
       <i/>
       <color rgb="FF7A6050"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
     </font>
     <font>
       <b/>
@@ -402,11 +417,6 @@
     </font>
     <font>
       <i/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF7A6050"/>
-      <sz val="9"/>
     </font>
     <font>
       <b/>
@@ -506,23 +516,25 @@
     <xf numFmtId="2" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -864,7 +876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -2137,45 +2149,45 @@
       <c r="G70" s="7"/>
       <c r="H70" s="7"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A72" s="14" t="s">
+    <row r="71" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B72" s="14"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
-      <c r="G72" s="14"/>
-      <c r="H72" s="14"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A73" s="14" t="s">
+      <c r="B71" s="5"/>
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B73" s="14"/>
-      <c r="C73" s="14"/>
-      <c r="D73" s="14"/>
-      <c r="E73" s="14"/>
-      <c r="F73" s="14"/>
-      <c r="G73" s="14"/>
-      <c r="H73" s="14"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A74" s="14" t="s">
+      <c r="B72" s="8">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B74" s="14"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
-      <c r="G74" s="14"/>
-      <c r="H74" s="14"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B73" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B74" s="12">
+        <f>IF(OR(B72="",B72=0),"",B73/B72)</f>
+      </c>
+    </row>
+    <row r="75" ht="42" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B75" s="14"/>
       <c r="C75" s="14"/>
@@ -2185,20 +2197,68 @@
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A76" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="14"/>
-      <c r="F76" s="14"/>
-      <c r="G76" s="14"/>
-      <c r="H76" s="14"/>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B77" s="2"/>
+      <c r="C77" s="2"/>
+      <c r="D77" s="2"/>
+      <c r="E77" s="2"/>
+      <c r="F77" s="2"/>
+      <c r="G77" s="2"/>
+      <c r="H77" s="2"/>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B78" s="2"/>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
+      <c r="E78" s="2"/>
+      <c r="F78" s="2"/>
+      <c r="G78" s="2"/>
+      <c r="H78" s="2"/>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B79" s="2"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2"/>
+      <c r="E79" s="2"/>
+      <c r="F79" s="2"/>
+      <c r="G79" s="2"/>
+      <c r="H79" s="2"/>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B80" s="2"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2"/>
+      <c r="E80" s="2"/>
+      <c r="F80" s="2"/>
+      <c r="G80" s="2"/>
+      <c r="H80" s="2"/>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B81" s="2"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
+      <c r="E81" s="2"/>
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+      <c r="H81" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="18">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
@@ -2210,14 +2270,16 @@
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A63:H63"/>
     <mergeCell ref="A68:H68"/>
-    <mergeCell ref="A72:H72"/>
-    <mergeCell ref="A73:H73"/>
-    <mergeCell ref="A74:H74"/>
+    <mergeCell ref="A71:H71"/>
     <mergeCell ref="A75:H75"/>
-    <mergeCell ref="A76:H76"/>
+    <mergeCell ref="A77:H77"/>
+    <mergeCell ref="A78:H78"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="A80:H80"/>
+    <mergeCell ref="A81:H81"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2234,7 +2296,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -2248,7 +2310,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2262,45 +2324,45 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J3" s="16" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D4" s="8">
         <v>332</v>
@@ -2324,13 +2386,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D5" s="8">
         <v>327</v>
@@ -2354,13 +2416,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D6" s="8">
         <v>314</v>
@@ -2384,13 +2446,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D7" s="8">
         <v>306</v>
@@ -2414,13 +2476,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D8" s="8">
         <v>302</v>
@@ -2444,13 +2506,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D9" s="8">
         <v>295</v>
@@ -2474,13 +2536,13 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D10" s="8">
         <v>294</v>
@@ -2504,7 +2566,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="I12" s="20">
         <f>SUM(I4:I10)</f>
@@ -2512,25 +2574,25 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="I13" s="22">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="14"/>
+      <c r="A14" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2539,6 +2601,6 @@
     <mergeCell ref="A14:J14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Shutdown 28.09.: Optin-Seiten Datum 25.10. + Formulare, Salespage-Programm final, Aufwaermmail Leroy, Webinar-Transkript
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/webinar-gelaende/launch-auswertung-gelaende.xlsx
+++ b/outputs/webinar-gelaende/launch-auswertung-gelaende.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="124">
   <si>
     <t>Launch-Auswertung Gelände-Webinar</t>
   </si>
@@ -26,6 +26,9 @@
     <t>Aug 2026</t>
   </si>
   <si>
+    <t>Sep 2026</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -44,6 +47,9 @@
     <t>23.08.2026</t>
   </si>
   <si>
+    <t>27.09.2026</t>
+  </si>
+  <si>
     <t>Webinar-Uhrzeit</t>
   </si>
   <si>
@@ -119,7 +125,7 @@
     <t>Anwesend am Ende</t>
   </si>
   <si>
-    <t>VERKAUF — PROGRAMM (549 €)</t>
+    <t>VERKAUF — PROGRAMM (549 €, ab Okt-Runde 749 €)</t>
   </si>
   <si>
     <t>Programm-Käufe gesamt (Stück)</t>
@@ -273,6 +279,9 @@
   </si>
   <si>
     <t>Show-up nach Quelle = Näherung über „Zoom-Link geklickt" (4 Erinnerungs-/Live-Mails, dedupliziert, gegen die Anmeldelisten gematcht; Bot-/Scanner-Klicks fallen automatisch raus). Klick ist etwas lockerer als „bis zum Schluss dabei". Verifiziert plausibel: Proxy-Gesamt 42,9 % liegt knapp über der echten Gesamt-Show-up von 40,5 %.</t>
+  </si>
+  <si>
+    <t>SEP 2026 (Stand 28.09.): Anmeldungen aus Devine-Tags „gelände webinar 09.26" (82) + „gelände webinar ads 09.26" (71), 3 doppelt → 150. Ad-Spend 535,32 € (Meta-API: Sandkasten August 14.–17.09. 224,39 € · Interessen September 17.–22.09. 206,79 € · Broad September 17.–22.09. 104,14 €); Budget ab 22.09. aufgebraucht → 5 Tage vor dem Webinar keine neuen Ads-Anmeldungen. Live 47 = Zoom-Namen bereinigt (72 Einwahlen). Pitch-Start nach 59 Min (Aug nach 75 Min). Show-up nach Quelle diesmal ohne Link-Klick-Proxy; Namensabgleich Zoom↔Devine: von 21 zuordenbaren Personen 18 organisch, 3 Ads. Preis diese Runde weiter 549 € (Klarna ab 49 €/Monat), Schnellentscheider-Bonus Tiergespräch bis Mo 28.09. Verkäufe/VIP/Checkout folgen nach Cart-Close Do 01.10.</t>
   </si>
   <si>
     <t>Sales-Mail-Auswertung Gelände-Webinar (Aug 2026)</t>
@@ -479,7 +488,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -516,6 +525,7 @@
     <xf numFmtId="2" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -876,7 +886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -918,24 +928,24 @@
         <v>4</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -947,12 +957,14 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>8</v>
+      </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
@@ -961,12 +973,14 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="7"/>
+        <v>10</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>11</v>
+      </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -975,12 +989,14 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="7"/>
+        <v>13</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>13</v>
+      </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
@@ -989,7 +1005,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1001,12 +1017,14 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B9" s="8">
         <v>165</v>
       </c>
-      <c r="C9" s="8"/>
+      <c r="C9" s="8">
+        <v>82</v>
+      </c>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
@@ -1015,12 +1033,14 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B10" s="8">
         <v>192</v>
       </c>
-      <c r="C10" s="8"/>
+      <c r="C10" s="8">
+        <v>71</v>
+      </c>
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
@@ -1029,12 +1049,14 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11" s="8">
         <v>9</v>
       </c>
-      <c r="C11" s="8"/>
+      <c r="C11" s="8">
+        <v>3</v>
+      </c>
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
@@ -1043,7 +1065,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B12" s="9">
         <f>B9+B10-B11</f>
@@ -1069,12 +1091,14 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B13" s="10">
         <v>1124.64</v>
       </c>
-      <c r="C13" s="10"/>
+      <c r="C13" s="10">
+        <v>535.32</v>
+      </c>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -1083,7 +1107,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B14" s="11">
         <f>IF(B10=0,"",B13/B10)</f>
@@ -1109,7 +1133,7 @@
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1121,7 +1145,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B16" s="8">
         <v>318</v>
@@ -1135,7 +1159,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B17" s="12">
         <f>IF(OR(B16="",B16=0),"",B9/B16)</f>
@@ -1161,7 +1185,7 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B18" s="8">
         <v>882</v>
@@ -1175,7 +1199,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B19" s="12">
         <f>IF(OR(B18="",B18=0),"",B10/B18)</f>
@@ -1201,7 +1225,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B20" s="9">
         <f>B16+B18</f>
@@ -1227,7 +1251,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B21" s="12">
         <f>IF(OR(B20="",B20=0),"",B12/B20)</f>
@@ -1253,7 +1277,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -1265,7 +1289,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B23" s="12">
         <f>IF(OR(B22="",B22=0),"",B32/B22)</f>
@@ -1291,7 +1315,7 @@
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1303,12 +1327,14 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B25" s="8">
         <v>141</v>
       </c>
-      <c r="C25" s="8"/>
+      <c r="C25" s="8">
+        <v>47</v>
+      </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
@@ -1317,7 +1343,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B26" s="12">
         <f>IF(B12=0,"",B25/B12)</f>
@@ -1343,12 +1369,14 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B27" s="8">
         <v>98</v>
       </c>
-      <c r="C27" s="8"/>
+      <c r="C27" s="8">
+        <v>87</v>
+      </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
@@ -1357,12 +1385,14 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B28" s="8">
         <v>110</v>
       </c>
-      <c r="C28" s="8"/>
+      <c r="C28" s="8">
+        <v>35</v>
+      </c>
       <c r="D28" s="8"/>
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
@@ -1371,7 +1401,7 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B29" s="12">
         <f>IF(B25=0,"",B28/B25)</f>
@@ -1397,12 +1427,14 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B30" s="8">
         <v>27</v>
       </c>
-      <c r="C30" s="8"/>
+      <c r="C30" s="8">
+        <v>13</v>
+      </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
@@ -1411,7 +1443,7 @@
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -1423,7 +1455,7 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B32" s="8">
         <v>7</v>
@@ -1437,7 +1469,7 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B33" s="10">
         <v>3415.98</v>
@@ -1451,7 +1483,7 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B34" s="8">
         <v>2</v>
@@ -1465,7 +1497,7 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B35" s="10">
         <v>922.68</v>
@@ -1479,7 +1511,7 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B36" s="8">
         <v>5</v>
@@ -1493,7 +1525,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B37" s="10">
         <v>2493.3</v>
@@ -1507,7 +1539,7 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B38" s="8">
         <v>5</v>
@@ -1521,7 +1553,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B39" s="8">
         <v>2</v>
@@ -1535,7 +1567,7 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B40" s="8">
         <v>4</v>
@@ -1549,7 +1581,7 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B41" s="8">
         <v>4</v>
@@ -1563,7 +1595,7 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -1575,7 +1607,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B43" s="9">
         <f>IF(B32="","",B32-IF(B42="",0,B42))</f>
@@ -1601,7 +1633,7 @@
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
@@ -1613,7 +1645,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B45" s="8">
         <v>15</v>
@@ -1627,7 +1659,7 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B46" s="10">
         <v>112.48</v>
@@ -1641,7 +1673,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B47" s="8">
         <v>21</v>
@@ -1655,7 +1687,7 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B48" s="10">
         <v>157.46</v>
@@ -1669,7 +1701,7 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B49" s="9">
         <f>B45+B47</f>
@@ -1695,7 +1727,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B50" s="11">
         <f>B46+B48</f>
@@ -1721,7 +1753,7 @@
     </row>
     <row r="51" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
@@ -1733,7 +1765,7 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B52" s="11">
         <f>N(B35)+N(B46)</f>
@@ -1759,7 +1791,7 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B53" s="11">
         <f>N(B37)+N(B48)</f>
@@ -1785,7 +1817,7 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B54" s="11">
         <f>N(B33)+N(B50)</f>
@@ -1811,7 +1843,7 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B55" s="11">
         <f>IF(OR(B32="",B32=0),"",B33/B32)</f>
@@ -1837,7 +1869,7 @@
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B56" s="12">
         <f>IF(OR(B32="",B12=0),"",B32/B12)</f>
@@ -1863,7 +1895,7 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B57" s="12">
         <f>IF(OR(B32="",B25=0),"",B32/B25)</f>
@@ -1889,7 +1921,7 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B58" s="12">
         <f>IF(OR(B32="",B28=0),"",B32/B28)</f>
@@ -1915,7 +1947,7 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B59" s="13">
         <f>IF(OR(B34="",B13="",B13=0),"",B52/B13)</f>
@@ -1941,7 +1973,7 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B60" s="13">
         <f>IF(OR(B33="",B13="",B13=0),"",B54/B13)</f>
@@ -1967,7 +1999,7 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B61" s="11">
         <f>IF(OR(B34="",B34=0,B13=""),"",B13/B34)</f>
@@ -1993,7 +2025,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B62" s="11">
         <f>IF(OR(B33="",B13=""),"",B54-B13)</f>
@@ -2019,7 +2051,7 @@
     </row>
     <row r="63" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
@@ -2031,7 +2063,7 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B64" s="8">
         <v>81</v>
@@ -2045,7 +2077,7 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B65" s="8">
         <v>72</v>
@@ -2059,7 +2091,7 @@
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B66" s="12">
         <f>IF(OR(B64="",B9=0),"",B64/B9)</f>
@@ -2085,7 +2117,7 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B67" s="12">
         <f>IF(OR(B65="",B10=0),"",B65/B10)</f>
@@ -2111,7 +2143,7 @@
     </row>
     <row r="68" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
@@ -2123,10 +2155,10 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C69" s="7"/>
       <c r="D69" s="7"/>
@@ -2137,10 +2169,10 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C70" s="7"/>
       <c r="D70" s="7"/>
@@ -2151,7 +2183,7 @@
     </row>
     <row r="71" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B71" s="5"/>
       <c r="C71" s="5"/>
@@ -2163,7 +2195,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B72" s="8">
         <v>37</v>
@@ -2171,35 +2203,38 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B73" s="8">
         <v>7</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B74" s="12">
         <f>IF(OR(B72="",B72=0),"",B73/B72)</f>
       </c>
+      <c r="C74" s="14">
+        <f>IF(OR(C72="",C72=0),"",C73/C72)</f>
+      </c>
     </row>
     <row r="75" ht="42" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A75" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B75" s="14"/>
-      <c r="C75" s="14"/>
-      <c r="D75" s="14"/>
-      <c r="E75" s="14"/>
-      <c r="F75" s="14"/>
-      <c r="G75" s="14"/>
-      <c r="H75" s="14"/>
+      <c r="A75" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B75" s="15"/>
+      <c r="C75" s="15"/>
+      <c r="D75" s="15"/>
+      <c r="E75" s="15"/>
+      <c r="F75" s="15"/>
+      <c r="G75" s="15"/>
+      <c r="H75" s="15"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -2211,7 +2246,7 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -2223,7 +2258,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -2235,7 +2270,7 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -2247,7 +2282,7 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -2257,8 +2292,20 @@
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
     </row>
+    <row r="82" ht="60" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B82" s="2"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
+      <c r="E82" s="2"/>
+      <c r="F82" s="2"/>
+      <c r="G82" s="2"/>
+      <c r="H82" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
@@ -2277,6 +2324,7 @@
     <mergeCell ref="A79:H79"/>
     <mergeCell ref="A80:H80"/>
     <mergeCell ref="A81:H81"/>
+    <mergeCell ref="A82:H82"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -2295,22 +2343,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
+      <c r="A1" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2324,45 +2372,45 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="E3" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="C3" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="D3" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="E3" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="F3" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="G3" s="17" t="s">
         <v>98</v>
       </c>
+      <c r="H3" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>100</v>
+      <c r="A4" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>103</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D4" s="8">
         <v>332</v>
@@ -2370,13 +2418,13 @@
       <c r="E4" s="8">
         <v>202</v>
       </c>
-      <c r="F4" s="19">
+      <c r="F4" s="20">
         <f>IF(OR(D4="",D4=0),"",E4/D4)</f>
       </c>
       <c r="G4" s="8">
         <v>36</v>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="20">
         <f>IF(OR(D4="",D4=0),"",G4/D4)</f>
       </c>
       <c r="I4" s="8">
@@ -2385,14 +2433,14 @@
       <c r="J4" s="8"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>103</v>
+      <c r="A5" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>106</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D5" s="8">
         <v>327</v>
@@ -2400,13 +2448,13 @@
       <c r="E5" s="8">
         <v>157</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="20">
         <f>IF(OR(D5="",D5=0),"",E5/D5)</f>
       </c>
       <c r="G5" s="8">
         <v>12</v>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="20">
         <f>IF(OR(D5="",D5=0),"",G5/D5)</f>
       </c>
       <c r="I5" s="8">
@@ -2415,14 +2463,14 @@
       <c r="J5" s="8"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>106</v>
+      <c r="A6" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>109</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D6" s="8">
         <v>314</v>
@@ -2430,13 +2478,13 @@
       <c r="E6" s="8">
         <v>138</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="20">
         <f>IF(OR(D6="",D6=0),"",E6/D6)</f>
       </c>
       <c r="G6" s="8">
         <v>13</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="20">
         <f>IF(OR(D6="",D6=0),"",G6/D6)</f>
       </c>
       <c r="I6" s="8">
@@ -2445,14 +2493,14 @@
       <c r="J6" s="8"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>108</v>
+      <c r="A7" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>111</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D7" s="8">
         <v>306</v>
@@ -2460,13 +2508,13 @@
       <c r="E7" s="8">
         <v>140</v>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="20">
         <f>IF(OR(D7="",D7=0),"",E7/D7)</f>
       </c>
       <c r="G7" s="8">
         <v>6</v>
       </c>
-      <c r="H7" s="19">
+      <c r="H7" s="20">
         <f>IF(OR(D7="",D7=0),"",G7/D7)</f>
       </c>
       <c r="I7" s="8">
@@ -2475,14 +2523,14 @@
       <c r="J7" s="8"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>111</v>
+      <c r="A8" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>114</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D8" s="8">
         <v>302</v>
@@ -2490,13 +2538,13 @@
       <c r="E8" s="8">
         <v>144</v>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="20">
         <f>IF(OR(D8="",D8=0),"",E8/D8)</f>
       </c>
       <c r="G8" s="8">
         <v>10</v>
       </c>
-      <c r="H8" s="19">
+      <c r="H8" s="20">
         <f>IF(OR(D8="",D8=0),"",G8/D8)</f>
       </c>
       <c r="I8" s="8">
@@ -2505,14 +2553,14 @@
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>113</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>114</v>
+      <c r="A9" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>117</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D9" s="8">
         <v>295</v>
@@ -2520,13 +2568,13 @@
       <c r="E9" s="8">
         <v>97</v>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="20">
         <f>IF(OR(D9="",D9=0),"",E9/D9)</f>
       </c>
       <c r="G9" s="8">
         <v>5</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="20">
         <f>IF(OR(D9="",D9=0),"",G9/D9)</f>
       </c>
       <c r="I9" s="8">
@@ -2535,14 +2583,14 @@
       <c r="J9" s="8"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>117</v>
+      <c r="A10" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>120</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D10" s="8">
         <v>294</v>
@@ -2550,13 +2598,13 @@
       <c r="E10" s="8">
         <v>86</v>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="20">
         <f>IF(OR(D10="",D10=0),"",E10/D10)</f>
       </c>
       <c r="G10" s="8">
         <v>7</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="20">
         <f>IF(OR(D10="",D10=0),"",G10/D10)</f>
       </c>
       <c r="I10" s="8">
@@ -2565,24 +2613,24 @@
       <c r="J10" s="8"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="I12" s="20">
+      <c r="A12" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="I12" s="21">
         <f>SUM(I4:I10)</f>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
-        <v>119</v>
-      </c>
-      <c r="I13" s="22">
+      <c r="A13" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="I13" s="23">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>

</xml_diff>

<commit_message>
Shutdown: Devine DND-Wiederherstellung und Listen-Aufraeumen dokumentiert, Kontaktlisten per .gitignore lokal gehalten, offene Aenderungen gesichert
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/webinar-gelaende/launch-auswertung-gelaende.xlsx
+++ b/outputs/webinar-gelaende/launch-auswertung-gelaende.xlsx
@@ -7,13 +7,14 @@
     <sheet sheetId="1" name="Launch-Auswertung" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Sales-Mails" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Fazit" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Downsell-Mails" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="165">
   <si>
     <t>Launch-Auswertung Gelände-Webinar</t>
   </si>
@@ -475,6 +476,39 @@
   </si>
   <si>
     <t>Kleine, durch einen Automationsfehler gebremste Runde. 150 Anmeldungen (82 org / 71 Ads, CPL 7,54 €), 47 live (31 % Show-up), 2 Programm-Käufe (1.010,34 € netto) + 5 VIP + 1 Freiarbeitskurs-Cross-Sell, Gewinn grob 512,82 €, Gesamt-ROAS 1,96. Kernlehre: Die Vorfreude-/Reminder-Automation lief nur organisch → Ads-Show-up nur 2,8 % statt 34,1 % organisch (behoben für den 25.10.). Überarbeitete Verkaufsmails: Klickrate in 6 von 7 Mails gehalten/gesteigert, Reframe „Hilft mir das beim Ausreiten?" (M6) + neue Bonus-Mail (M7) = Keeper. Höhere Abmelderate (kleine, mehrfach angeschriebene Liste) = gesunde Selbstselektion.</t>
+  </si>
+  <si>
+    <t>Downsell-Auswertung Gelände-Paket (Sep 2026)</t>
+  </si>
+  <si>
+    <t>Downsell-Strecke an die Programm-Nicht-Käufer (Bundle Gelände-Schlüssel + sicher meistern, 199 €). Zahlen aus Devine. Käufe = Gelände-Paket-Bestellungen (ThriveCart).</t>
+  </si>
+  <si>
+    <t>Downsell Mail 1</t>
+  </si>
+  <si>
+    <t>Mo 05.10.</t>
+  </si>
+  <si>
+    <t>Downsell Mail 2</t>
+  </si>
+  <si>
+    <t>Di 06.10.</t>
+  </si>
+  <si>
+    <t>Downsell Mail 3</t>
+  </si>
+  <si>
+    <t>Mi 07.10. vorm.</t>
+  </si>
+  <si>
+    <t>Downsell Mail 4 Last Call</t>
+  </si>
+  <si>
+    <t>Mi 07.10. abends</t>
+  </si>
+  <si>
+    <t>Abmeldungen gesamt (Downsell)</t>
   </si>
 </sst>
 </file>
@@ -485,7 +519,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -547,6 +581,11 @@
       <color rgb="FFFFFFFF"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -593,7 +632,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -656,6 +695,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -663,6 +703,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2521,7 +2562,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -3140,6 +3181,47 @@
       <c r="I29">
         <v>10</v>
       </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="19"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="15"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="28"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="28"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F34" s="27"/>
+      <c r="H34" s="27"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F35" s="27"/>
+      <c r="H35" s="27"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F36" s="27"/>
+      <c r="H36" s="27"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F37" s="27"/>
+      <c r="H37" s="27"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="16"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3165,20 +3247,20 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="30" t="s">
         <v>151</v>
       </c>
     </row>
@@ -3189,7 +3271,7 @@
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="31" t="s">
         <v>152</v>
       </c>
     </row>
@@ -3200,7 +3282,7 @@
       <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="31" t="s">
         <v>153</v>
       </c>
     </row>
@@ -3209,6 +3291,222 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="H3" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="J3" s="30" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4">
+        <v>89</v>
+      </c>
+      <c r="E4">
+        <v>23</v>
+      </c>
+      <c r="F4" s="27">
+        <v>0.25842696629213485</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" s="27">
+        <v>0.011235955056179775</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>159</v>
+      </c>
+      <c r="D5">
+        <v>87</v>
+      </c>
+      <c r="E5">
+        <v>21</v>
+      </c>
+      <c r="F5" s="27">
+        <v>0.2413793103448276</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5" s="27">
+        <v>0.034482758620689655</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D6">
+        <v>87</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+      <c r="F6" s="27">
+        <v>0.22988505747126436</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6" s="27">
+        <v>0.034482758620689655</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7">
+        <v>110</v>
+      </c>
+      <c r="E7">
+        <v>27</v>
+      </c>
+      <c r="F7" s="27">
+        <v>0.24545454545454545</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7" s="27">
+        <v>0.01818181818181818</v>
+      </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="I9">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Shutdown: ManyChat-Kontext (Facebook-Versionen, Erinnerungen), Webinar- und Call-Auswertungen gesichert
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/webinar-gelaende/launch-auswertung-gelaende.xlsx
+++ b/outputs/webinar-gelaende/launch-auswertung-gelaende.xlsx
@@ -3,6 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11055"/>
+  </bookViews>
   <sheets>
     <sheet sheetId="1" name="Launch-Auswertung" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Sales-Mails" state="visible" r:id="rId5"/>
@@ -14,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="166">
   <si>
     <t>Launch-Auswertung Gelände-Webinar</t>
   </si>
@@ -29,6 +32,9 @@
   </si>
   <si>
     <t>Sep 2026</t>
+  </si>
+  <si>
+    <t>Okt 2026</t>
   </si>
   <si>
     <t/>
@@ -519,7 +525,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -531,60 +537,75 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="16"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <i/>
       <color rgb="FF7A6050"/>
       <sz val="9"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF7B3F28"/>
       <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <color rgb="FF2C2C2C"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <i/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="14"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF2C2C2C"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <i/>
       <color rgb="FF7A6050"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF7B3F28"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="13"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="12"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -632,7 +653,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -649,6 +670,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -690,20 +714,20 @@
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1044,13 +1068,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H87"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="9.140625"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="8" width="13.5" customWidth="1"/>
+    <col min="2" max="8" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="26.1" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1088,21 +1112,21 @@
         <v>5</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -1114,15 +1138,17 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="7"/>
+        <v>9</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
@@ -1130,15 +1156,17 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="7"/>
+        <v>12</v>
+      </c>
+      <c r="D6" s="8">
+        <v>46320</v>
+      </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
@@ -1146,15 +1174,17 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>14</v>
+      </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -1162,7 +1192,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1174,123 +1204,140 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="8">
+        <v>16</v>
+      </c>
+      <c r="B9" s="9">
         <v>165</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="9">
         <v>82</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
+      <c r="D9" s="9">
+        <v>87</v>
+      </c>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="8">
+        <v>17</v>
+      </c>
+      <c r="B10" s="9">
         <v>192</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="9">
         <v>71</v>
       </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
+      <c r="D10" s="9">
+        <v>35</v>
+      </c>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="8">
+        <v>18</v>
+      </c>
+      <c r="B11" s="9">
         <v>9</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="9">
         <v>3</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
+      <c r="D11" s="9">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="9">
-        <f>B9+B10-B11</f>
-      </c>
-      <c r="C12" s="9">
-        <f>C9+C10-C11</f>
-      </c>
-      <c r="D12" s="9">
+        <v>19</v>
+      </c>
+      <c r="B12" s="10">
+        <f t="shared" ref="B12:H12" si="0">B9+B10-B11</f>
+        <v>348</v>
+      </c>
+      <c r="C12" s="10">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+      <c r="D12" s="10">
         <f>D9+D10-D11</f>
       </c>
-      <c r="E12" s="9">
-        <f>E9+E10-E11</f>
-      </c>
-      <c r="F12" s="9">
-        <f>F9+F10-F11</f>
-      </c>
-      <c r="G12" s="9">
-        <f>G9+G10-G11</f>
-      </c>
-      <c r="H12" s="9">
-        <f>H9+H10-H11</f>
+      <c r="E12" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F12" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H12" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="10">
+        <v>20</v>
+      </c>
+      <c r="B13" s="11">
         <v>1124.64</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="11">
         <v>535.32</v>
       </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
+      <c r="D13" s="11">
+        <v>204.24</v>
+      </c>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="11">
-        <f>IF(B10=0,"",B13/B10)</f>
-      </c>
-      <c r="C14" s="11">
-        <f>IF(C10=0,"",C13/C10)</f>
-      </c>
-      <c r="D14" s="11">
-        <f>IF(D10=0,"",D13/D10)</f>
-      </c>
-      <c r="E14" s="11">
-        <f>IF(E10=0,"",E13/E10)</f>
-      </c>
-      <c r="F14" s="11">
-        <f>IF(F10=0,"",F13/F10)</f>
-      </c>
-      <c r="G14" s="11">
-        <f>IF(G10=0,"",G13/G10)</f>
-      </c>
-      <c r="H14" s="11">
-        <f>IF(H10=0,"",H13/H10)</f>
+        <v>21</v>
+      </c>
+      <c r="B14" s="12">
+        <f t="shared" ref="B14:H14" si="1">IF(B10=0,"",B13/B10)</f>
+        <v>5.857500000000001</v>
+      </c>
+      <c r="C14" s="12">
+        <f t="shared" si="1"/>
+        <v>7.539718309859156</v>
+      </c>
+      <c r="D14" s="12">
+        <f t="shared" si="1"/>
+        <v>5.053714285714285</v>
+      </c>
+      <c r="E14" s="12">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="F14" s="12">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="G14" s="12">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H14" s="12">
+        <f t="shared" si="1"/>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1302,183 +1349,201 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="8">
+        <v>23</v>
+      </c>
+      <c r="B16" s="9">
         <v>318</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="9">
         <v>163</v>
       </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
+      <c r="D16" s="9">
+        <v>131</v>
+      </c>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="12">
-        <f>IF(OR(B16="",B16=0),"",B9/B16)</f>
-      </c>
-      <c r="C17" s="12">
-        <f>IF(OR(C16="",C16=0),"",C9/C16)</f>
-      </c>
-      <c r="D17" s="12">
-        <f>IF(OR(D16="",D16=0),"",D9/D16)</f>
-      </c>
-      <c r="E17" s="12">
-        <f>IF(OR(E16="",E16=0),"",E9/E16)</f>
-      </c>
-      <c r="F17" s="12">
-        <f>IF(OR(F16="",F16=0),"",F9/F16)</f>
-      </c>
-      <c r="G17" s="12">
-        <f>IF(OR(G16="",G16=0),"",G9/G16)</f>
-      </c>
-      <c r="H17" s="12">
-        <f>IF(OR(H16="",H16=0),"",H9/H16)</f>
+        <v>24</v>
+      </c>
+      <c r="B17" s="13">
+        <f t="shared" ref="B17:H17" si="2">IF(OR(B16="",B16=0),"",B9/B16)</f>
+        <v>0.5188679245283019</v>
+      </c>
+      <c r="C17" s="13">
+        <f t="shared" si="2"/>
+        <v>0.5030674846625767</v>
+      </c>
+      <c r="D17" s="13">
+        <f t="shared" si="2"/>
+      </c>
+      <c r="E17" s="13">
+        <f t="shared" si="2"/>
+      </c>
+      <c r="F17" s="13">
+        <f t="shared" si="2"/>
+      </c>
+      <c r="G17" s="13">
+        <f t="shared" si="2"/>
+      </c>
+      <c r="H17" s="13">
+        <f t="shared" si="2"/>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="8">
+        <v>25</v>
+      </c>
+      <c r="B18" s="9">
         <v>882</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="9">
         <v>345</v>
       </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
+      <c r="D18" s="9">
+        <v>233</v>
+      </c>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="12">
-        <f>IF(OR(B18="",B18=0),"",B10/B18)</f>
-      </c>
-      <c r="C19" s="12">
-        <f>IF(OR(C18="",C18=0),"",C10/C18)</f>
-      </c>
-      <c r="D19" s="12">
-        <f>IF(OR(D18="",D18=0),"",D10/D18)</f>
-      </c>
-      <c r="E19" s="12">
-        <f>IF(OR(E18="",E18=0),"",E10/E18)</f>
-      </c>
-      <c r="F19" s="12">
-        <f>IF(OR(F18="",F18=0),"",F10/F18)</f>
-      </c>
-      <c r="G19" s="12">
-        <f>IF(OR(G18="",G18=0),"",G10/G18)</f>
-      </c>
-      <c r="H19" s="12">
-        <f>IF(OR(H18="",H18=0),"",H10/H18)</f>
+        <v>26</v>
+      </c>
+      <c r="B19" s="13">
+        <f t="shared" ref="B19:H19" si="3">IF(OR(B18="",B18=0),"",B10/B18)</f>
+        <v>0.21768707482993196</v>
+      </c>
+      <c r="C19" s="13">
+        <f t="shared" si="3"/>
+        <v>0.20579710144927535</v>
+      </c>
+      <c r="D19" s="13">
+        <f t="shared" si="3"/>
+      </c>
+      <c r="E19" s="13">
+        <f t="shared" si="3"/>
+      </c>
+      <c r="F19" s="13">
+        <f t="shared" si="3"/>
+      </c>
+      <c r="G19" s="13">
+        <f t="shared" si="3"/>
+      </c>
+      <c r="H19" s="13">
+        <f t="shared" si="3"/>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="9">
-        <f>B16+B18</f>
-      </c>
-      <c r="C20" s="9">
-        <f>C16+C18</f>
-      </c>
-      <c r="D20" s="9">
-        <f>D16+D18</f>
-      </c>
-      <c r="E20" s="9">
-        <f>E16+E18</f>
-      </c>
-      <c r="F20" s="9">
-        <f>F16+F18</f>
-      </c>
-      <c r="G20" s="9">
-        <f>G16+G18</f>
-      </c>
-      <c r="H20" s="9">
-        <f>H16+H18</f>
+        <v>27</v>
+      </c>
+      <c r="B20" s="10">
+        <f t="shared" ref="B20:H20" si="4">B16+B18</f>
+        <v>1200</v>
+      </c>
+      <c r="C20" s="10">
+        <f t="shared" si="4"/>
+        <v>508</v>
+      </c>
+      <c r="D20" s="10">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E20" s="10">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F20" s="10">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="10">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="H20" s="10">
+        <f t="shared" si="4"/>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="12">
-        <f>IF(OR(B20="",B20=0),"",B12/B20)</f>
-      </c>
-      <c r="C21" s="12">
-        <f>IF(OR(C20="",C20=0),"",C12/C20)</f>
-      </c>
-      <c r="D21" s="12">
-        <f>IF(OR(D20="",D20=0),"",D12/D20)</f>
-      </c>
-      <c r="E21" s="12">
-        <f>IF(OR(E20="",E20=0),"",E12/E20)</f>
-      </c>
-      <c r="F21" s="12">
-        <f>IF(OR(F20="",F20=0),"",F12/F20)</f>
-      </c>
-      <c r="G21" s="12">
-        <f>IF(OR(G20="",G20=0),"",G12/G20)</f>
-      </c>
-      <c r="H21" s="12">
-        <f>IF(OR(H20="",H20=0),"",H12/H20)</f>
+        <v>28</v>
+      </c>
+      <c r="B21" s="13">
+        <f t="shared" ref="B21:H21" si="5">IF(OR(B20="",B20=0),"",B12/B20)</f>
+        <v>0.29</v>
+      </c>
+      <c r="C21" s="13">
+        <f t="shared" si="5"/>
+        <v>0.2952755905511811</v>
+      </c>
+      <c r="D21" s="13">
+        <f t="shared" si="5"/>
+      </c>
+      <c r="E21" s="13">
+        <f t="shared" si="5"/>
+      </c>
+      <c r="F21" s="13">
+        <f t="shared" si="5"/>
+      </c>
+      <c r="G21" s="13">
+        <f t="shared" si="5"/>
+      </c>
+      <c r="H21" s="13">
+        <f t="shared" si="5"/>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8">
+        <v>29</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9">
         <v>16</v>
       </c>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B23" s="12">
-        <f>IF(OR(B22="",B22=0),"",B32/B22)</f>
-      </c>
-      <c r="C23" s="12">
-        <f>IF(OR(C22="",C22=0),"",C32/C22)</f>
-      </c>
-      <c r="D23" s="12">
-        <f>IF(OR(D22="",D22=0),"",D32/D22)</f>
-      </c>
-      <c r="E23" s="12">
-        <f>IF(OR(E22="",E22=0),"",E32/E22)</f>
-      </c>
-      <c r="F23" s="12">
-        <f>IF(OR(F22="",F22=0),"",F32/F22)</f>
-      </c>
-      <c r="G23" s="12">
-        <f>IF(OR(G22="",G22=0),"",G32/G22)</f>
-      </c>
-      <c r="H23" s="12">
-        <f>IF(OR(H22="",H22=0),"",H32/H22)</f>
+        <v>30</v>
+      </c>
+      <c r="B23" s="13">
+        <f t="shared" ref="B23:H23" si="6">IF(OR(B22="",B22=0),"",B32/B22)</f>
+      </c>
+      <c r="C23" s="13">
+        <f t="shared" si="6"/>
+        <v>0.125</v>
+      </c>
+      <c r="D23" s="13">
+        <f t="shared" si="6"/>
+      </c>
+      <c r="E23" s="13">
+        <f t="shared" si="6"/>
+      </c>
+      <c r="F23" s="13">
+        <f t="shared" si="6"/>
+      </c>
+      <c r="G23" s="13">
+        <f t="shared" si="6"/>
+      </c>
+      <c r="H23" s="13">
+        <f t="shared" si="6"/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1490,123 +1555,136 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="8">
+        <v>32</v>
+      </c>
+      <c r="B25" s="9">
         <v>141</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="9">
         <v>47</v>
       </c>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
+      <c r="D25" s="9">
+        <v>39</v>
+      </c>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B26" s="12">
-        <f>IF(B12=0,"",B25/B12)</f>
-      </c>
-      <c r="C26" s="12">
-        <f>IF(C12=0,"",C25/C12)</f>
-      </c>
-      <c r="D26" s="12">
-        <f>IF(D12=0,"",D25/D12)</f>
-      </c>
-      <c r="E26" s="12">
-        <f>IF(E12=0,"",E25/E12)</f>
-      </c>
-      <c r="F26" s="12">
-        <f>IF(F12=0,"",F25/F12)</f>
-      </c>
-      <c r="G26" s="12">
-        <f>IF(G12=0,"",G25/G12)</f>
-      </c>
-      <c r="H26" s="12">
-        <f>IF(H12=0,"",H25/H12)</f>
+        <v>33</v>
+      </c>
+      <c r="B26" s="13">
+        <f t="shared" ref="B26:H26" si="7">IF(B12=0,"",B25/B12)</f>
+        <v>0.4051724137931034</v>
+      </c>
+      <c r="C26" s="13">
+        <f t="shared" si="7"/>
+        <v>0.31333333333333335</v>
+      </c>
+      <c r="D26" s="13">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E26" s="13">
+        <f t="shared" si="7"/>
+      </c>
+      <c r="F26" s="13">
+        <f t="shared" si="7"/>
+      </c>
+      <c r="G26" s="13">
+        <f t="shared" si="7"/>
+      </c>
+      <c r="H26" s="13">
+        <f t="shared" si="7"/>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" s="8">
+        <v>34</v>
+      </c>
+      <c r="B27" s="9">
         <v>98</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="9">
         <v>87</v>
       </c>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
+      <c r="D27" s="9">
+        <v>83</v>
+      </c>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B28" s="8">
+        <v>35</v>
+      </c>
+      <c r="B28" s="9">
         <v>110</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="9">
         <v>35</v>
       </c>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
+      <c r="D28" s="9">
+        <v>25</v>
+      </c>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B29" s="12">
-        <f>IF(B25=0,"",B28/B25)</f>
-      </c>
-      <c r="C29" s="12">
-        <f>IF(C25=0,"",C28/C25)</f>
-      </c>
-      <c r="D29" s="12">
-        <f>IF(D25=0,"",D28/D25)</f>
-      </c>
-      <c r="E29" s="12">
-        <f>IF(E25=0,"",E28/E25)</f>
-      </c>
-      <c r="F29" s="12">
-        <f>IF(F25=0,"",F28/F25)</f>
-      </c>
-      <c r="G29" s="12">
-        <f>IF(G25=0,"",G28/G25)</f>
-      </c>
-      <c r="H29" s="12">
-        <f>IF(H25=0,"",H28/H25)</f>
+        <v>36</v>
+      </c>
+      <c r="B29" s="13">
+        <f t="shared" ref="B29:H29" si="8">IF(B25=0,"",B28/B25)</f>
+        <v>0.7801418439716312</v>
+      </c>
+      <c r="C29" s="13">
+        <f t="shared" si="8"/>
+        <v>0.7446808510638298</v>
+      </c>
+      <c r="D29" s="13">
+        <f t="shared" si="8"/>
+      </c>
+      <c r="E29" s="13">
+        <f t="shared" si="8"/>
+      </c>
+      <c r="F29" s="13">
+        <f t="shared" si="8"/>
+      </c>
+      <c r="G29" s="13">
+        <f t="shared" si="8"/>
+      </c>
+      <c r="H29" s="13">
+        <f t="shared" si="8"/>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="8">
+        <v>37</v>
+      </c>
+      <c r="B30" s="9">
         <v>27</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C30" s="9">
         <v>13</v>
       </c>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
+      <c r="D30" s="9">
+        <v>14</v>
+      </c>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -1618,207 +1696,209 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B32" s="8">
+        <v>39</v>
+      </c>
+      <c r="B32" s="9">
         <v>7</v>
       </c>
-      <c r="C32" s="8">
+      <c r="C32" s="9">
         <v>2</v>
       </c>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="10">
+        <v>40</v>
+      </c>
+      <c r="B33" s="11">
         <v>3415.98</v>
       </c>
-      <c r="C33" s="10">
+      <c r="C33" s="11">
         <v>1010.34</v>
       </c>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B34" s="8">
+        <v>41</v>
+      </c>
+      <c r="B34" s="9">
         <v>2</v>
       </c>
-      <c r="C34" s="8">
-        <v>0</v>
-      </c>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
+      <c r="C34" s="9">
+        <v>0</v>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" s="10">
+        <v>42</v>
+      </c>
+      <c r="B35" s="11">
         <v>922.68</v>
       </c>
-      <c r="C35" s="10">
-        <v>0</v>
-      </c>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
+      <c r="C35" s="11">
+        <v>0</v>
+      </c>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B36" s="8">
+        <v>43</v>
+      </c>
+      <c r="B36" s="9">
         <v>5</v>
       </c>
-      <c r="C36" s="8">
+      <c r="C36" s="9">
         <v>2</v>
       </c>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B37" s="10">
+        <v>44</v>
+      </c>
+      <c r="B37" s="11">
         <v>2493.3</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="11">
         <v>1010.34</v>
       </c>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B38" s="8">
+        <v>45</v>
+      </c>
+      <c r="B38" s="9">
         <v>5</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="9">
         <v>2</v>
       </c>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B39" s="8">
+        <v>46</v>
+      </c>
+      <c r="B39" s="9">
         <v>2</v>
       </c>
-      <c r="C39" s="8">
-        <v>0</v>
-      </c>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
+      <c r="C39" s="9">
+        <v>0</v>
+      </c>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B40" s="8">
+        <v>47</v>
+      </c>
+      <c r="B40" s="9">
         <v>4</v>
       </c>
-      <c r="C40" s="8">
+      <c r="C40" s="9">
         <v>2</v>
       </c>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B41" s="8">
+        <v>48</v>
+      </c>
+      <c r="B41" s="9">
         <v>4</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C41" s="9">
         <v>1</v>
       </c>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8">
-        <v>0</v>
-      </c>
-      <c r="D42" s="8"/>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="8"/>
+        <v>49</v>
+      </c>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9">
+        <v>0</v>
+      </c>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B43" s="9">
-        <f>IF(B32="","",B32-IF(B42="",0,B42))</f>
-      </c>
-      <c r="C43" s="9">
-        <f>IF(C32="","",C32-IF(C42="",0,C42))</f>
-      </c>
-      <c r="D43" s="9">
-        <f>IF(D32="","",D32-IF(D42="",0,D42))</f>
-      </c>
-      <c r="E43" s="9">
-        <f>IF(E32="","",E32-IF(E42="",0,E42))</f>
-      </c>
-      <c r="F43" s="9">
-        <f>IF(F32="","",F32-IF(F42="",0,F42))</f>
-      </c>
-      <c r="G43" s="9">
-        <f>IF(G32="","",G32-IF(G42="",0,G42))</f>
-      </c>
-      <c r="H43" s="9">
-        <f>IF(H32="","",H32-IF(H42="",0,H42))</f>
+        <v>50</v>
+      </c>
+      <c r="B43" s="10">
+        <f t="shared" ref="B43:H43" si="9">IF(B32="","",B32-IF(B42="",0,B42))</f>
+        <v>7</v>
+      </c>
+      <c r="C43" s="10">
+        <f t="shared" si="9"/>
+        <v>2</v>
+      </c>
+      <c r="D43" s="10">
+        <f t="shared" si="9"/>
+      </c>
+      <c r="E43" s="10">
+        <f t="shared" si="9"/>
+      </c>
+      <c r="F43" s="10">
+        <f t="shared" si="9"/>
+      </c>
+      <c r="G43" s="10">
+        <f t="shared" si="9"/>
+      </c>
+      <c r="H43" s="10">
+        <f t="shared" si="9"/>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
@@ -1830,123 +1910,145 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B45" s="8">
+        <v>52</v>
+      </c>
+      <c r="B45" s="9">
         <v>15</v>
       </c>
-      <c r="C45" s="8">
-        <v>0</v>
-      </c>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="8"/>
+      <c r="C45" s="9">
+        <v>0</v>
+      </c>
+      <c r="D45" s="9">
+        <v>3</v>
+      </c>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B46" s="10">
+        <v>53</v>
+      </c>
+      <c r="B46" s="11">
         <v>112.48</v>
       </c>
-      <c r="C46" s="10">
-        <v>0</v>
-      </c>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10"/>
+      <c r="C46" s="11">
+        <v>0</v>
+      </c>
+      <c r="D46" s="11">
+        <v>24.06</v>
+      </c>
+      <c r="E46" s="11"/>
+      <c r="F46" s="11"/>
+      <c r="G46" s="11"/>
+      <c r="H46" s="11"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B47" s="8">
+        <v>54</v>
+      </c>
+      <c r="B47" s="9">
         <v>21</v>
       </c>
-      <c r="C47" s="8">
+      <c r="C47" s="9">
         <v>5</v>
       </c>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
+      <c r="D47" s="9">
+        <v>1</v>
+      </c>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B48" s="10">
+        <v>55</v>
+      </c>
+      <c r="B48" s="11">
         <v>157.46</v>
       </c>
-      <c r="C48" s="10">
+      <c r="C48" s="11">
         <v>37.8</v>
       </c>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
+      <c r="D48" s="11">
+        <v>7.44</v>
+      </c>
+      <c r="E48" s="11"/>
+      <c r="F48" s="11"/>
+      <c r="G48" s="11"/>
+      <c r="H48" s="11"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B49" s="9">
-        <f>B45+B47</f>
-      </c>
-      <c r="C49" s="9">
-        <f>C45+C47</f>
-      </c>
-      <c r="D49" s="9">
-        <f>D45+D47</f>
-      </c>
-      <c r="E49" s="9">
-        <f>E45+E47</f>
-      </c>
-      <c r="F49" s="9">
-        <f>F45+F47</f>
-      </c>
-      <c r="G49" s="9">
-        <f>G45+G47</f>
-      </c>
-      <c r="H49" s="9">
-        <f>H45+H47</f>
+        <v>56</v>
+      </c>
+      <c r="B49" s="10">
+        <f t="shared" ref="B49:H50" si="10">B45+B47</f>
+        <v>36</v>
+      </c>
+      <c r="C49" s="10">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
+      <c r="D49" s="10">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="E49" s="10">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="F49" s="10">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="G49" s="10">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="H49" s="10">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B50" s="11">
-        <f>B46+B48</f>
-      </c>
-      <c r="C50" s="11">
-        <f>C46+C48</f>
-      </c>
-      <c r="D50" s="11">
-        <f>D46+D48</f>
-      </c>
-      <c r="E50" s="11">
-        <f>E46+E48</f>
-      </c>
-      <c r="F50" s="11">
-        <f>F46+F48</f>
-      </c>
-      <c r="G50" s="11">
-        <f>G46+G48</f>
-      </c>
-      <c r="H50" s="11">
-        <f>H46+H48</f>
+        <v>57</v>
+      </c>
+      <c r="B50" s="12">
+        <f t="shared" si="10"/>
+        <v>269.94</v>
+      </c>
+      <c r="C50" s="12">
+        <f t="shared" si="10"/>
+        <v>37.8</v>
+      </c>
+      <c r="D50" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="E50" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="F50" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="G50" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="H50" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
@@ -1958,293 +2060,329 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B52" s="11">
-        <f>N(B35)+N(B46)</f>
-      </c>
-      <c r="C52" s="11">
-        <f>N(C35)+N(C46)</f>
-      </c>
-      <c r="D52" s="11">
-        <f>N(D35)+N(D46)</f>
-      </c>
-      <c r="E52" s="11">
-        <f>N(E35)+N(E46)</f>
-      </c>
-      <c r="F52" s="11">
-        <f>N(F35)+N(F46)</f>
-      </c>
-      <c r="G52" s="11">
-        <f>N(G35)+N(G46)</f>
-      </c>
-      <c r="H52" s="11">
-        <f>N(H35)+N(H46)</f>
+        <v>59</v>
+      </c>
+      <c r="B52" s="12">
+        <f t="shared" ref="B52:H52" si="11">N(B35)+N(B46)</f>
+        <v>1035.1599999999999</v>
+      </c>
+      <c r="C52" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="D52" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="E52" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F52" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G52" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="H52" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B53" s="11">
-        <f>N(B37)+N(B48)</f>
-      </c>
-      <c r="C53" s="11">
-        <f>N(C37)+N(C48)</f>
-      </c>
-      <c r="D53" s="11">
-        <f>N(D37)+N(D48)</f>
-      </c>
-      <c r="E53" s="11">
-        <f>N(E37)+N(E48)</f>
-      </c>
-      <c r="F53" s="11">
-        <f>N(F37)+N(F48)</f>
-      </c>
-      <c r="G53" s="11">
-        <f>N(G37)+N(G48)</f>
-      </c>
-      <c r="H53" s="11">
-        <f>N(H37)+N(H48)</f>
+        <v>60</v>
+      </c>
+      <c r="B53" s="12">
+        <f t="shared" ref="B53:H53" si="12">N(B37)+N(B48)</f>
+        <v>2650.76</v>
+      </c>
+      <c r="C53" s="12">
+        <f t="shared" si="12"/>
+        <v>1048.14</v>
+      </c>
+      <c r="D53" s="12">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="E53" s="12">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F53" s="12">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G53" s="12">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="H53" s="12">
+        <f t="shared" si="12"/>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B54" s="11">
-        <f>N(B33)+N(B50)</f>
-      </c>
-      <c r="C54" s="11">
-        <f>N(C33)+N(C50)</f>
-      </c>
-      <c r="D54" s="11">
-        <f>N(D33)+N(D50)</f>
-      </c>
-      <c r="E54" s="11">
-        <f>N(E33)+N(E50)</f>
-      </c>
-      <c r="F54" s="11">
-        <f>N(F33)+N(F50)</f>
-      </c>
-      <c r="G54" s="11">
-        <f>N(G33)+N(G50)</f>
-      </c>
-      <c r="H54" s="11">
-        <f>N(H33)+N(H50)</f>
+        <v>61</v>
+      </c>
+      <c r="B54" s="12">
+        <f t="shared" ref="B54:H54" si="13">N(B33)+N(B50)</f>
+        <v>3685.92</v>
+      </c>
+      <c r="C54" s="12">
+        <f t="shared" si="13"/>
+        <v>1048.14</v>
+      </c>
+      <c r="D54" s="12">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="E54" s="12">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F54" s="12">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G54" s="12">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="H54" s="12">
+        <f t="shared" si="13"/>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B55" s="11">
-        <f>IF(OR(B32="",B32=0),"",B33/B32)</f>
-      </c>
-      <c r="C55" s="11">
-        <f>IF(OR(C32="",C32=0),"",C33/C32)</f>
-      </c>
-      <c r="D55" s="11">
-        <f>IF(OR(D32="",D32=0),"",D33/D32)</f>
-      </c>
-      <c r="E55" s="11">
-        <f>IF(OR(E32="",E32=0),"",E33/E32)</f>
-      </c>
-      <c r="F55" s="11">
-        <f>IF(OR(F32="",F32=0),"",F33/F32)</f>
-      </c>
-      <c r="G55" s="11">
-        <f>IF(OR(G32="",G32=0),"",G33/G32)</f>
-      </c>
-      <c r="H55" s="11">
-        <f>IF(OR(H32="",H32=0),"",H33/H32)</f>
+        <v>62</v>
+      </c>
+      <c r="B55" s="12">
+        <f t="shared" ref="B55:H55" si="14">IF(OR(B32="",B32=0),"",B33/B32)</f>
+        <v>487.9971428571429</v>
+      </c>
+      <c r="C55" s="12">
+        <f t="shared" si="14"/>
+        <v>505.17</v>
+      </c>
+      <c r="D55" s="12">
+        <f t="shared" si="14"/>
+      </c>
+      <c r="E55" s="12">
+        <f t="shared" si="14"/>
+      </c>
+      <c r="F55" s="12">
+        <f t="shared" si="14"/>
+      </c>
+      <c r="G55" s="12">
+        <f t="shared" si="14"/>
+      </c>
+      <c r="H55" s="12">
+        <f t="shared" si="14"/>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B56" s="12">
-        <f>IF(OR(B32="",B12=0),"",B32/B12)</f>
-      </c>
-      <c r="C56" s="12">
-        <f>IF(OR(C32="",C12=0),"",C32/C12)</f>
-      </c>
-      <c r="D56" s="12">
-        <f>IF(OR(D32="",D12=0),"",D32/D12)</f>
-      </c>
-      <c r="E56" s="12">
-        <f>IF(OR(E32="",E12=0),"",E32/E12)</f>
-      </c>
-      <c r="F56" s="12">
-        <f>IF(OR(F32="",F12=0),"",F32/F12)</f>
-      </c>
-      <c r="G56" s="12">
-        <f>IF(OR(G32="",G12=0),"",G32/G12)</f>
-      </c>
-      <c r="H56" s="12">
-        <f>IF(OR(H32="",H12=0),"",H32/H12)</f>
+        <v>63</v>
+      </c>
+      <c r="B56" s="13">
+        <f t="shared" ref="B56:H56" si="15">IF(OR(B32="",B12=0),"",B32/B12)</f>
+        <v>0.020114942528735632</v>
+      </c>
+      <c r="C56" s="13">
+        <f t="shared" si="15"/>
+        <v>0.013333333333333334</v>
+      </c>
+      <c r="D56" s="13">
+        <f t="shared" si="15"/>
+      </c>
+      <c r="E56" s="13">
+        <f t="shared" si="15"/>
+      </c>
+      <c r="F56" s="13">
+        <f t="shared" si="15"/>
+      </c>
+      <c r="G56" s="13">
+        <f t="shared" si="15"/>
+      </c>
+      <c r="H56" s="13">
+        <f t="shared" si="15"/>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B57" s="12">
-        <f>IF(OR(B32="",B25=0),"",B32/B25)</f>
-      </c>
-      <c r="C57" s="12">
-        <f>IF(OR(C32="",C25=0),"",C32/C25)</f>
-      </c>
-      <c r="D57" s="12">
-        <f>IF(OR(D32="",D25=0),"",D32/D25)</f>
-      </c>
-      <c r="E57" s="12">
-        <f>IF(OR(E32="",E25=0),"",E32/E25)</f>
-      </c>
-      <c r="F57" s="12">
-        <f>IF(OR(F32="",F25=0),"",F32/F25)</f>
-      </c>
-      <c r="G57" s="12">
-        <f>IF(OR(G32="",G25=0),"",G32/G25)</f>
-      </c>
-      <c r="H57" s="12">
-        <f>IF(OR(H32="",H25=0),"",H32/H25)</f>
+        <v>64</v>
+      </c>
+      <c r="B57" s="13">
+        <f t="shared" ref="B57:H57" si="16">IF(OR(B32="",B25=0),"",B32/B25)</f>
+        <v>0.04964539007092199</v>
+      </c>
+      <c r="C57" s="13">
+        <f t="shared" si="16"/>
+        <v>0.0425531914893617</v>
+      </c>
+      <c r="D57" s="13">
+        <f t="shared" si="16"/>
+      </c>
+      <c r="E57" s="13">
+        <f t="shared" si="16"/>
+      </c>
+      <c r="F57" s="13">
+        <f t="shared" si="16"/>
+      </c>
+      <c r="G57" s="13">
+        <f t="shared" si="16"/>
+      </c>
+      <c r="H57" s="13">
+        <f t="shared" si="16"/>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B58" s="12">
-        <f>IF(OR(B32="",B28=0),"",B32/B28)</f>
-      </c>
-      <c r="C58" s="12">
-        <f>IF(OR(C32="",C28=0),"",C32/C28)</f>
-      </c>
-      <c r="D58" s="12">
-        <f>IF(OR(D32="",D28=0),"",D32/D28)</f>
-      </c>
-      <c r="E58" s="12">
-        <f>IF(OR(E32="",E28=0),"",E32/E28)</f>
-      </c>
-      <c r="F58" s="12">
-        <f>IF(OR(F32="",F28=0),"",F32/F28)</f>
-      </c>
-      <c r="G58" s="12">
-        <f>IF(OR(G32="",G28=0),"",G32/G28)</f>
-      </c>
-      <c r="H58" s="12">
-        <f>IF(OR(H32="",H28=0),"",H32/H28)</f>
+        <v>65</v>
+      </c>
+      <c r="B58" s="13">
+        <f t="shared" ref="B58:H58" si="17">IF(OR(B32="",B28=0),"",B32/B28)</f>
+        <v>0.06363636363636363</v>
+      </c>
+      <c r="C58" s="13">
+        <f t="shared" si="17"/>
+        <v>0.05714285714285714</v>
+      </c>
+      <c r="D58" s="13">
+        <f t="shared" si="17"/>
+      </c>
+      <c r="E58" s="13">
+        <f t="shared" si="17"/>
+      </c>
+      <c r="F58" s="13">
+        <f t="shared" si="17"/>
+      </c>
+      <c r="G58" s="13">
+        <f t="shared" si="17"/>
+      </c>
+      <c r="H58" s="13">
+        <f t="shared" si="17"/>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B59" s="13">
-        <f>IF(OR(B34="",B13="",B13=0),"",B52/B13)</f>
-      </c>
-      <c r="C59" s="13">
-        <f>IF(OR(C34="",C13="",C13=0),"",C52/C13)</f>
-      </c>
-      <c r="D59" s="13">
-        <f>IF(OR(D34="",D13="",D13=0),"",D52/D13)</f>
-      </c>
-      <c r="E59" s="13">
-        <f>IF(OR(E34="",E13="",E13=0),"",E52/E13)</f>
-      </c>
-      <c r="F59" s="13">
-        <f>IF(OR(F34="",F13="",F13=0),"",F52/F13)</f>
-      </c>
-      <c r="G59" s="13">
-        <f>IF(OR(G34="",G13="",G13=0),"",G52/G13)</f>
-      </c>
-      <c r="H59" s="13">
-        <f>IF(OR(H34="",H13="",H13=0),"",H52/H13)</f>
+        <v>66</v>
+      </c>
+      <c r="B59" s="14">
+        <f t="shared" ref="B59:H59" si="18">IF(OR(B34="",B13="",B13=0),"",B52/B13)</f>
+        <v>0.9204367619860575</v>
+      </c>
+      <c r="C59" s="14">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="D59" s="14">
+        <f t="shared" si="18"/>
+      </c>
+      <c r="E59" s="14">
+        <f t="shared" si="18"/>
+      </c>
+      <c r="F59" s="14">
+        <f t="shared" si="18"/>
+      </c>
+      <c r="G59" s="14">
+        <f t="shared" si="18"/>
+      </c>
+      <c r="H59" s="14">
+        <f t="shared" si="18"/>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B60" s="13">
-        <f>IF(OR(B33="",B13="",B13=0),"",B54/B13)</f>
-      </c>
-      <c r="C60" s="13">
-        <f>IF(OR(C33="",C13="",C13=0),"",C54/C13)</f>
-      </c>
-      <c r="D60" s="13">
-        <f>IF(OR(D33="",D13="",D13=0),"",D54/D13)</f>
-      </c>
-      <c r="E60" s="13">
-        <f>IF(OR(E33="",E13="",E13=0),"",E54/E13)</f>
-      </c>
-      <c r="F60" s="13">
-        <f>IF(OR(F33="",F13="",F13=0),"",F54/F13)</f>
-      </c>
-      <c r="G60" s="13">
-        <f>IF(OR(G33="",G13="",G13=0),"",G54/G13)</f>
-      </c>
-      <c r="H60" s="13">
-        <f>IF(OR(H33="",H13="",H13=0),"",H54/H13)</f>
+        <v>67</v>
+      </c>
+      <c r="B60" s="14">
+        <f t="shared" ref="B60:H60" si="19">IF(OR(B33="",B13="",B13=0),"",B54/B13)</f>
+        <v>3.2774221084080235</v>
+      </c>
+      <c r="C60" s="14">
+        <f t="shared" si="19"/>
+        <v>1.9579690652320108</v>
+      </c>
+      <c r="D60" s="14">
+        <f t="shared" si="19"/>
+      </c>
+      <c r="E60" s="14">
+        <f t="shared" si="19"/>
+      </c>
+      <c r="F60" s="14">
+        <f t="shared" si="19"/>
+      </c>
+      <c r="G60" s="14">
+        <f t="shared" si="19"/>
+      </c>
+      <c r="H60" s="14">
+        <f t="shared" si="19"/>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B61" s="11">
-        <f>IF(OR(B34="",B34=0,B13=""),"",B13/B34)</f>
-      </c>
-      <c r="C61" s="11">
-        <f>IF(OR(C34="",C34=0,C13=""),"",C13/C34)</f>
-      </c>
-      <c r="D61" s="11">
-        <f>IF(OR(D34="",D34=0,D13=""),"",D13/D34)</f>
-      </c>
-      <c r="E61" s="11">
-        <f>IF(OR(E34="",E34=0,E13=""),"",E13/E34)</f>
-      </c>
-      <c r="F61" s="11">
-        <f>IF(OR(F34="",F34=0,F13=""),"",F13/F34)</f>
-      </c>
-      <c r="G61" s="11">
-        <f>IF(OR(G34="",G34=0,G13=""),"",G13/G34)</f>
-      </c>
-      <c r="H61" s="11">
-        <f>IF(OR(H34="",H34=0,H13=""),"",H13/H34)</f>
+        <v>68</v>
+      </c>
+      <c r="B61" s="12">
+        <f t="shared" ref="B61:H61" si="20">IF(OR(B34="",B34=0,B13=""),"",B13/B34)</f>
+        <v>562.32</v>
+      </c>
+      <c r="C61" s="12">
+        <f t="shared" si="20"/>
+      </c>
+      <c r="D61" s="12">
+        <f t="shared" si="20"/>
+      </c>
+      <c r="E61" s="12">
+        <f t="shared" si="20"/>
+      </c>
+      <c r="F61" s="12">
+        <f t="shared" si="20"/>
+      </c>
+      <c r="G61" s="12">
+        <f t="shared" si="20"/>
+      </c>
+      <c r="H61" s="12">
+        <f t="shared" si="20"/>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B62" s="11">
-        <f>IF(OR(B33="",B13=""),"",B54-B13)</f>
-      </c>
-      <c r="C62" s="11">
-        <f>IF(OR(C33="",C13=""),"",C54-C13)</f>
-      </c>
-      <c r="D62" s="11">
-        <f>IF(OR(D33="",D13=""),"",D54-D13)</f>
-      </c>
-      <c r="E62" s="11">
-        <f>IF(OR(E33="",E13=""),"",E54-E13)</f>
-      </c>
-      <c r="F62" s="11">
-        <f>IF(OR(F33="",F13=""),"",F54-F13)</f>
-      </c>
-      <c r="G62" s="11">
-        <f>IF(OR(G33="",G13=""),"",G54-G13)</f>
-      </c>
-      <c r="H62" s="11">
-        <f>IF(OR(H33="",H13=""),"",H54-H13)</f>
+        <v>69</v>
+      </c>
+      <c r="B62" s="12">
+        <f t="shared" ref="B62:H62" si="21">IF(OR(B33="",B13=""),"",B54-B13)</f>
+        <v>2561.2799999999997</v>
+      </c>
+      <c r="C62" s="12">
+        <f t="shared" si="21"/>
+        <v>512.82</v>
+      </c>
+      <c r="D62" s="12">
+        <f t="shared" si="21"/>
+      </c>
+      <c r="E62" s="12">
+        <f t="shared" si="21"/>
+      </c>
+      <c r="F62" s="12">
+        <f t="shared" si="21"/>
+      </c>
+      <c r="G62" s="12">
+        <f t="shared" si="21"/>
+      </c>
+      <c r="H62" s="12">
+        <f t="shared" si="21"/>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
@@ -2256,91 +2394,99 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B64" s="8">
+        <v>71</v>
+      </c>
+      <c r="B64" s="9">
         <v>81</v>
       </c>
-      <c r="C64" s="8">
+      <c r="C64" s="9">
         <v>28</v>
       </c>
-      <c r="D64" s="8"/>
-      <c r="E64" s="8"/>
-      <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
+      <c r="D64" s="9">
+        <v>19</v>
+      </c>
+      <c r="E64" s="9"/>
+      <c r="F64" s="9"/>
+      <c r="G64" s="9"/>
+      <c r="H64" s="9"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B65" s="8">
         <v>72</v>
       </c>
-      <c r="C65" s="8">
+      <c r="B65" s="9">
+        <v>72</v>
+      </c>
+      <c r="C65" s="9">
         <v>2</v>
       </c>
-      <c r="D65" s="8"/>
-      <c r="E65" s="8"/>
-      <c r="F65" s="8"/>
-      <c r="G65" s="8"/>
-      <c r="H65" s="8"/>
+      <c r="D65" s="9">
+        <v>10</v>
+      </c>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B66" s="12">
-        <f>IF(OR(B64="",B9=0),"",B64/B9)</f>
-      </c>
-      <c r="C66" s="12">
-        <f>IF(OR(C64="",C9=0),"",C64/C9)</f>
-      </c>
-      <c r="D66" s="12">
-        <f>IF(OR(D64="",D9=0),"",D64/D9)</f>
-      </c>
-      <c r="E66" s="12">
-        <f>IF(OR(E64="",E9=0),"",E64/E9)</f>
-      </c>
-      <c r="F66" s="12">
-        <f>IF(OR(F64="",F9=0),"",F64/F9)</f>
-      </c>
-      <c r="G66" s="12">
-        <f>IF(OR(G64="",G9=0),"",G64/G9)</f>
-      </c>
-      <c r="H66" s="12">
-        <f>IF(OR(H64="",H9=0),"",H64/H9)</f>
+        <v>73</v>
+      </c>
+      <c r="B66" s="13">
+        <f t="shared" ref="B66:H67" si="22">IF(OR(B64="",B9=0),"",B64/B9)</f>
+        <v>0.4909090909090909</v>
+      </c>
+      <c r="C66" s="13">
+        <f t="shared" si="22"/>
+        <v>0.34146341463414637</v>
+      </c>
+      <c r="D66" s="13">
+        <f t="shared" si="22"/>
+      </c>
+      <c r="E66" s="13">
+        <f t="shared" si="22"/>
+      </c>
+      <c r="F66" s="13">
+        <f t="shared" si="22"/>
+      </c>
+      <c r="G66" s="13">
+        <f t="shared" si="22"/>
+      </c>
+      <c r="H66" s="13">
+        <f t="shared" si="22"/>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B67" s="12">
-        <f>IF(OR(B65="",B10=0),"",B65/B10)</f>
-      </c>
-      <c r="C67" s="12">
-        <f>IF(OR(C65="",C10=0),"",C65/C10)</f>
-      </c>
-      <c r="D67" s="12">
-        <f>IF(OR(D65="",D10=0),"",D65/D10)</f>
-      </c>
-      <c r="E67" s="12">
-        <f>IF(OR(E65="",E10=0),"",E65/E10)</f>
-      </c>
-      <c r="F67" s="12">
-        <f>IF(OR(F65="",F10=0),"",F65/F10)</f>
-      </c>
-      <c r="G67" s="12">
-        <f>IF(OR(G65="",G10=0),"",G65/G10)</f>
-      </c>
-      <c r="H67" s="12">
-        <f>IF(OR(H65="",H10=0),"",H65/H10)</f>
+        <v>74</v>
+      </c>
+      <c r="B67" s="13">
+        <f t="shared" si="22"/>
+        <v>0.375</v>
+      </c>
+      <c r="C67" s="13">
+        <f t="shared" si="22"/>
+        <v>0.028169014084507043</v>
+      </c>
+      <c r="D67" s="13">
+        <f t="shared" si="22"/>
+      </c>
+      <c r="E67" s="13">
+        <f t="shared" si="22"/>
+      </c>
+      <c r="F67" s="13">
+        <f t="shared" si="22"/>
+      </c>
+      <c r="G67" s="13">
+        <f t="shared" si="22"/>
+      </c>
+      <c r="H67" s="13">
+        <f t="shared" si="22"/>
       </c>
     </row>
     <row r="68" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
@@ -2352,10 +2498,10 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C69" s="7"/>
       <c r="D69" s="7"/>
@@ -2366,10 +2512,10 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C70" s="7"/>
       <c r="D70" s="7"/>
@@ -2380,7 +2526,7 @@
     </row>
     <row r="71" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B71" s="5"/>
       <c r="C71" s="5"/>
@@ -2392,9 +2538,9 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B72" s="8">
+        <v>81</v>
+      </c>
+      <c r="B72" s="9">
         <v>37</v>
       </c>
       <c r="C72">
@@ -2403,41 +2549,46 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B73" s="8">
+        <v>82</v>
+      </c>
+      <c r="B73" s="9">
         <v>7</v>
       </c>
       <c r="C73">
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B74" s="12">
+        <v>83</v>
+      </c>
+      <c r="B74" s="13">
         <f>IF(OR(B72="",B72=0),"",B73/B72)</f>
-      </c>
-      <c r="C74" s="14">
+        <v>0.1891891891891892</v>
+      </c>
+      <c r="C74" s="15">
         <f>IF(OR(C72="",C72=0),"",C73/C72)</f>
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="D74" s="15">
+        <f>IF(OR(D72="",D72=0),"",D73/D72)</f>
       </c>
     </row>
     <row r="75" ht="42" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A75" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="B75" s="15"/>
-      <c r="C75" s="15"/>
-      <c r="D75" s="15"/>
-      <c r="E75" s="15"/>
-      <c r="F75" s="15"/>
-      <c r="G75" s="15"/>
-      <c r="H75" s="15"/>
+      <c r="A75" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B75" s="16"/>
+      <c r="C75" s="16"/>
+      <c r="D75" s="16"/>
+      <c r="E75" s="16"/>
+      <c r="F75" s="16"/>
+      <c r="G75" s="16"/>
+      <c r="H75" s="16"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -2449,7 +2600,7 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -2461,7 +2612,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -2473,7 +2624,7 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -2485,7 +2636,7 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -2497,7 +2648,7 @@
     </row>
     <row r="82" ht="60" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -2508,13 +2659,13 @@
       <c r="H82" s="2"/>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" s="16" t="s">
-        <v>90</v>
+      <c r="A84" s="17" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C85">
         <v>1</v>
@@ -2522,15 +2673,15 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>92</v>
-      </c>
-      <c r="C86" s="17">
+        <v>93</v>
+      </c>
+      <c r="C86" s="18">
         <v>81.51</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" s="18" t="s">
-        <v>93</v>
+      <c r="A87" s="19" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2563,7 +2714,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J40"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="9.140625"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -2572,22 +2723,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
+      <c r="A1" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2599,267 +2750,282 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="H3" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="J3" s="21" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D4" s="9">
+        <v>332</v>
+      </c>
+      <c r="E4" s="9">
+        <v>202</v>
+      </c>
+      <c r="F4" s="24">
+        <f t="shared" ref="F4:F10" si="0">IF(OR(D4="",D4=0),"",E4/D4)</f>
+        <v>0.608433734939759</v>
+      </c>
+      <c r="G4" s="9">
+        <v>36</v>
+      </c>
+      <c r="H4" s="24">
+        <f t="shared" ref="H4:H10" si="1">IF(OR(D4="",D4=0),"",G4/D4)</f>
+        <v>0.10843373493975904</v>
+      </c>
+      <c r="I4" s="9">
+        <v>4</v>
+      </c>
+      <c r="J4" s="9"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D5" s="9">
+        <v>327</v>
+      </c>
+      <c r="E5" s="9">
+        <v>157</v>
+      </c>
+      <c r="F5" s="24">
+        <f t="shared" si="0"/>
+        <v>0.4801223241590214</v>
+      </c>
+      <c r="G5" s="9">
+        <v>12</v>
+      </c>
+      <c r="H5" s="24">
+        <f t="shared" si="1"/>
+        <v>0.03669724770642202</v>
+      </c>
+      <c r="I5" s="9">
+        <v>9</v>
+      </c>
+      <c r="J5" s="9"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D6" s="9">
+        <v>314</v>
+      </c>
+      <c r="E6" s="9">
+        <v>138</v>
+      </c>
+      <c r="F6" s="24">
+        <f t="shared" si="0"/>
+        <v>0.4394904458598726</v>
+      </c>
+      <c r="G6" s="9">
+        <v>13</v>
+      </c>
+      <c r="H6" s="24">
+        <f t="shared" si="1"/>
+        <v>0.041401273885350316</v>
+      </c>
+      <c r="I6" s="9">
+        <v>3</v>
+      </c>
+      <c r="J6" s="9"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D7" s="9">
+        <v>306</v>
+      </c>
+      <c r="E7" s="9">
+        <v>140</v>
+      </c>
+      <c r="F7" s="24">
+        <f t="shared" si="0"/>
+        <v>0.45751633986928103</v>
+      </c>
+      <c r="G7" s="9">
+        <v>6</v>
+      </c>
+      <c r="H7" s="24">
+        <f t="shared" si="1"/>
+        <v>0.0196078431372549</v>
+      </c>
+      <c r="I7" s="9">
+        <v>5</v>
+      </c>
+      <c r="J7" s="9"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" s="9">
+        <v>302</v>
+      </c>
+      <c r="E8" s="9">
+        <v>144</v>
+      </c>
+      <c r="F8" s="24">
+        <f t="shared" si="0"/>
+        <v>0.4768211920529801</v>
+      </c>
+      <c r="G8" s="9">
+        <v>10</v>
+      </c>
+      <c r="H8" s="24">
+        <f t="shared" si="1"/>
+        <v>0.033112582781456956</v>
+      </c>
+      <c r="I8" s="9">
+        <v>3</v>
+      </c>
+      <c r="J8" s="9"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="9">
+        <v>295</v>
+      </c>
+      <c r="E9" s="9">
         <v>97</v>
       </c>
-      <c r="C3" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="E3" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="G3" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="H3" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="I3" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="J3" s="20" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="D4" s="8">
-        <v>332</v>
-      </c>
-      <c r="E4" s="8">
-        <v>202</v>
-      </c>
-      <c r="F4" s="23">
-        <f>IF(OR(D4="",D4=0),"",E4/D4)</f>
-      </c>
-      <c r="G4" s="8">
-        <v>36</v>
-      </c>
-      <c r="H4" s="23">
-        <f>IF(OR(D4="",D4=0),"",G4/D4)</f>
-      </c>
-      <c r="I4" s="8">
-        <v>4</v>
-      </c>
-      <c r="J4" s="8"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="D5" s="8">
-        <v>327</v>
-      </c>
-      <c r="E5" s="8">
-        <v>157</v>
-      </c>
-      <c r="F5" s="23">
-        <f>IF(OR(D5="",D5=0),"",E5/D5)</f>
-      </c>
-      <c r="G5" s="8">
-        <v>12</v>
-      </c>
-      <c r="H5" s="23">
-        <f>IF(OR(D5="",D5=0),"",G5/D5)</f>
-      </c>
-      <c r="I5" s="8">
-        <v>9</v>
-      </c>
-      <c r="J5" s="8"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>113</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="D6" s="8">
-        <v>314</v>
-      </c>
-      <c r="E6" s="8">
-        <v>138</v>
-      </c>
-      <c r="F6" s="23">
-        <f>IF(OR(D6="",D6=0),"",E6/D6)</f>
-      </c>
-      <c r="G6" s="8">
-        <v>13</v>
-      </c>
-      <c r="H6" s="23">
-        <f>IF(OR(D6="",D6=0),"",G6/D6)</f>
-      </c>
-      <c r="I6" s="8">
-        <v>3</v>
-      </c>
-      <c r="J6" s="8"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="D7" s="8">
-        <v>306</v>
-      </c>
-      <c r="E7" s="8">
-        <v>140</v>
-      </c>
-      <c r="F7" s="23">
-        <f>IF(OR(D7="",D7=0),"",E7/D7)</f>
-      </c>
-      <c r="G7" s="8">
-        <v>6</v>
-      </c>
-      <c r="H7" s="23">
-        <f>IF(OR(D7="",D7=0),"",G7/D7)</f>
-      </c>
-      <c r="I7" s="8">
+      <c r="F9" s="24">
+        <f t="shared" si="0"/>
+        <v>0.3288135593220339</v>
+      </c>
+      <c r="G9" s="9">
         <v>5</v>
       </c>
-      <c r="J7" s="8"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D8" s="8">
-        <v>302</v>
-      </c>
-      <c r="E8" s="8">
-        <v>144</v>
-      </c>
-      <c r="F8" s="23">
-        <f>IF(OR(D8="",D8=0),"",E8/D8)</f>
-      </c>
-      <c r="G8" s="8">
-        <v>10</v>
-      </c>
-      <c r="H8" s="23">
-        <f>IF(OR(D8="",D8=0),"",G8/D8)</f>
-      </c>
-      <c r="I8" s="8">
-        <v>3</v>
-      </c>
-      <c r="J8" s="8"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D9" s="8">
-        <v>295</v>
-      </c>
-      <c r="E9" s="8">
-        <v>97</v>
-      </c>
-      <c r="F9" s="23">
-        <f>IF(OR(D9="",D9=0),"",E9/D9)</f>
-      </c>
-      <c r="G9" s="8">
-        <v>5</v>
-      </c>
-      <c r="H9" s="23">
-        <f>IF(OR(D9="",D9=0),"",G9/D9)</f>
-      </c>
-      <c r="I9" s="8">
+      <c r="H9" s="24">
+        <f t="shared" si="1"/>
+        <v>0.01694915254237288</v>
+      </c>
+      <c r="I9" s="9">
         <v>1</v>
       </c>
-      <c r="J9" s="8"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B10" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D10" s="8">
+      <c r="D10" s="9">
         <v>294</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="9">
         <v>86</v>
       </c>
-      <c r="F10" s="23">
-        <f>IF(OR(D10="",D10=0),"",E10/D10)</f>
-      </c>
-      <c r="G10" s="8">
+      <c r="F10" s="24">
+        <f t="shared" si="0"/>
+        <v>0.2925170068027211</v>
+      </c>
+      <c r="G10" s="9">
         <v>7</v>
       </c>
-      <c r="H10" s="23">
-        <f>IF(OR(D10="",D10=0),"",G10/D10)</f>
-      </c>
-      <c r="I10" s="8">
+      <c r="H10" s="24">
+        <f t="shared" si="1"/>
+        <v>0.023809523809523808</v>
+      </c>
+      <c r="I10" s="9">
         <v>2</v>
       </c>
-      <c r="J10" s="8"/>
+      <c r="J10" s="9"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="I12" s="24">
+      <c r="A12" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="I12" s="25">
         <f>SUM(I4:I10)</f>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="I13" s="26">
+      <c r="A13" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="I13" s="27">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2871,75 +3037,75 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
+    <row r="16" ht="18.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+    </row>
+    <row r="18" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C18" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="C18" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="D18" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="E18" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="F18" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="H18" s="20" t="s">
+      <c r="G18" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="I18" s="20" t="s">
+      <c r="H18" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="20" t="s">
+      <c r="I18" s="21" t="s">
         <v>105</v>
+      </c>
+      <c r="J18" s="21" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C19" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D19">
         <v>145</v>
@@ -2947,14 +3113,16 @@
       <c r="E19">
         <v>69</v>
       </c>
-      <c r="F19" s="27">
-        <f>IF(OR(D19="",D19=0),"",E19/D19)</f>
+      <c r="F19" s="28">
+        <f t="shared" ref="F19:F26" si="2">IF(OR(D19="",D19=0),"",E19/D19)</f>
+        <v>0.47586206896551725</v>
       </c>
       <c r="G19">
         <v>10</v>
       </c>
-      <c r="H19" s="27">
-        <f>IF(OR(D19="",D19=0),"",G19/D19)</f>
+      <c r="H19" s="28">
+        <f t="shared" ref="H19:H26" si="3">IF(OR(D19="",D19=0),"",G19/D19)</f>
+        <v>0.06896551724137931</v>
       </c>
       <c r="I19">
         <v>5</v>
@@ -2962,13 +3130,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C20" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D20">
         <v>141</v>
@@ -2976,14 +3144,16 @@
       <c r="E20">
         <v>65</v>
       </c>
-      <c r="F20" s="27">
-        <f>IF(OR(D20="",D20=0),"",E20/D20)</f>
+      <c r="F20" s="28">
+        <f t="shared" si="2"/>
+        <v>0.46099290780141844</v>
       </c>
       <c r="G20">
         <v>6</v>
       </c>
-      <c r="H20" s="27">
-        <f>IF(OR(D20="",D20=0),"",G20/D20)</f>
+      <c r="H20" s="28">
+        <f t="shared" si="3"/>
+        <v>0.0425531914893617</v>
       </c>
       <c r="I20">
         <v>5</v>
@@ -2991,13 +3161,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" t="s">
+        <v>138</v>
+      </c>
+      <c r="C21" t="s">
         <v>136</v>
-      </c>
-      <c r="B21" t="s">
-        <v>137</v>
-      </c>
-      <c r="C21" t="s">
-        <v>135</v>
       </c>
       <c r="D21">
         <v>136</v>
@@ -3005,14 +3175,16 @@
       <c r="E21">
         <v>57</v>
       </c>
-      <c r="F21" s="27">
-        <f>IF(OR(D21="",D21=0),"",E21/D21)</f>
+      <c r="F21" s="28">
+        <f t="shared" si="2"/>
+        <v>0.41911764705882354</v>
       </c>
       <c r="G21">
         <v>7</v>
       </c>
-      <c r="H21" s="27">
-        <f>IF(OR(D21="",D21=0),"",G21/D21)</f>
+      <c r="H21" s="28">
+        <f t="shared" si="3"/>
+        <v>0.051470588235294115</v>
       </c>
       <c r="I21">
         <v>5</v>
@@ -3020,13 +3192,13 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C22" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D22">
         <v>130</v>
@@ -3034,14 +3206,16 @@
       <c r="E22">
         <v>59</v>
       </c>
-      <c r="F22" s="27">
-        <f>IF(OR(D22="",D22=0),"",E22/D22)</f>
+      <c r="F22" s="28">
+        <f t="shared" si="2"/>
+        <v>0.45384615384615384</v>
       </c>
       <c r="G22">
         <v>4</v>
       </c>
-      <c r="H22" s="27">
-        <f>IF(OR(D22="",D22=0),"",G22/D22)</f>
+      <c r="H22" s="28">
+        <f t="shared" si="3"/>
+        <v>0.03076923076923077</v>
       </c>
       <c r="I22">
         <v>3</v>
@@ -3049,13 +3223,13 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B23" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D23">
         <v>122</v>
@@ -3063,14 +3237,16 @@
       <c r="E23">
         <v>56</v>
       </c>
-      <c r="F23" s="27">
-        <f>IF(OR(D23="",D23=0),"",E23/D23)</f>
+      <c r="F23" s="28">
+        <f t="shared" si="2"/>
+        <v>0.45901639344262296</v>
       </c>
       <c r="G23">
         <v>4</v>
       </c>
-      <c r="H23" s="27">
-        <f>IF(OR(D23="",D23=0),"",G23/D23)</f>
+      <c r="H23" s="28">
+        <f t="shared" si="3"/>
+        <v>0.03278688524590164</v>
       </c>
       <c r="I23">
         <v>2</v>
@@ -3081,13 +3257,13 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C24" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D24">
         <v>119</v>
@@ -3095,14 +3271,16 @@
       <c r="E24">
         <v>39</v>
       </c>
-      <c r="F24" s="27">
-        <f>IF(OR(D24="",D24=0),"",E24/D24)</f>
+      <c r="F24" s="28">
+        <f t="shared" si="2"/>
+        <v>0.3277310924369748</v>
       </c>
       <c r="G24">
         <v>6</v>
       </c>
-      <c r="H24" s="27">
-        <f>IF(OR(D24="",D24=0),"",G24/D24)</f>
+      <c r="H24" s="28">
+        <f t="shared" si="3"/>
+        <v>0.05042016806722689</v>
       </c>
       <c r="I24">
         <v>3</v>
@@ -3110,13 +3288,13 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>146</v>
+      </c>
+      <c r="B25" t="s">
+        <v>147</v>
+      </c>
+      <c r="C25" t="s">
         <v>145</v>
-      </c>
-      <c r="B25" t="s">
-        <v>146</v>
-      </c>
-      <c r="C25" t="s">
-        <v>144</v>
       </c>
       <c r="D25">
         <v>116</v>
@@ -3124,14 +3302,16 @@
       <c r="E25">
         <v>44</v>
       </c>
-      <c r="F25" s="27">
-        <f>IF(OR(D25="",D25=0),"",E25/D25)</f>
+      <c r="F25" s="28">
+        <f t="shared" si="2"/>
+        <v>0.3793103448275862</v>
       </c>
       <c r="G25">
         <v>3</v>
       </c>
-      <c r="H25" s="27">
-        <f>IF(OR(D25="",D25=0),"",G25/D25)</f>
+      <c r="H25" s="28">
+        <f t="shared" si="3"/>
+        <v>0.02586206896551724</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -3139,13 +3319,13 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B26" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C26" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D26">
         <v>115</v>
@@ -3153,75 +3333,77 @@
       <c r="E26">
         <v>35</v>
       </c>
-      <c r="F26" s="27">
-        <f>IF(OR(D26="",D26=0),"",E26/D26)</f>
+      <c r="F26" s="28">
+        <f t="shared" si="2"/>
+        <v>0.30434782608695654</v>
       </c>
       <c r="G26">
         <v>1</v>
       </c>
-      <c r="H26" s="27">
-        <f>IF(OR(D26="",D26=0),"",G26/D26)</f>
+      <c r="H26" s="28">
+        <f t="shared" si="3"/>
+        <v>0.008695652173913044</v>
       </c>
       <c r="I26">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
-        <v>125</v>
+      <c r="A28" s="17" t="s">
+        <v>126</v>
       </c>
       <c r="I28">
         <f>SUM(I19:I26)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
-        <v>126</v>
+      <c r="A29" s="17" t="s">
+        <v>127</v>
       </c>
       <c r="I29">
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="19"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="15"/>
+    <row r="31" ht="18.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="20"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="16"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="28"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="28"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F34" s="27"/>
-      <c r="H34" s="27"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F35" s="27"/>
-      <c r="H35" s="27"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F36" s="27"/>
-      <c r="H36" s="27"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F37" s="27"/>
-      <c r="H37" s="27"/>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="16"/>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
+      <c r="A33" s="29"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+      <c r="J33" s="29"/>
+    </row>
+    <row r="34" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F34" s="28"/>
+      <c r="H34" s="28"/>
+    </row>
+    <row r="35" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F35" s="28"/>
+      <c r="H35" s="28"/>
+    </row>
+    <row r="36" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F36" s="28"/>
+      <c r="H36" s="28"/>
+    </row>
+    <row r="37" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F37" s="28"/>
+      <c r="H37" s="28"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="17"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3239,7 +3421,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="9.140625"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -3247,43 +3429,43 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
+      <c r="A1" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="B3" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="30" t="s">
+      <c r="A3" s="31" t="s">
         <v>151</v>
       </c>
+      <c r="B3" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="4" ht="90" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="17" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="31" t="s">
-        <v>152</v>
+        <v>11</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="5" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>153</v>
+        <v>12</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -3298,82 +3480,82 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="9.140625"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
-        <v>154</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
+    <row r="1" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="33" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
-        <v>155</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
+      <c r="A2" s="32" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" s="30" t="s">
+      <c r="A3" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>98</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="C3" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="E3" s="30" t="s">
+      <c r="D3" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="E3" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="G3" s="30" t="s">
+      <c r="F3" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="G3" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="I3" s="30" t="s">
+      <c r="H3" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="J3" s="30" t="s">
+      <c r="I3" s="31" t="s">
         <v>105</v>
+      </c>
+      <c r="J3" s="31" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D4">
         <v>89</v>
@@ -3381,31 +3563,31 @@
       <c r="E4">
         <v>23</v>
       </c>
-      <c r="F4" s="27">
+      <c r="F4" s="28">
         <v>0.25842696629213485</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="28">
         <v>0.011235955056179775</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D5">
         <v>87</v>
@@ -3413,31 +3595,31 @@
       <c r="E5">
         <v>21</v>
       </c>
-      <c r="F5" s="27">
+      <c r="F5" s="28">
         <v>0.2413793103448276</v>
       </c>
       <c r="G5">
         <v>3</v>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="28">
         <v>0.034482758620689655</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D6">
         <v>87</v>
@@ -3445,31 +3627,31 @@
       <c r="E6">
         <v>20</v>
       </c>
-      <c r="F6" s="27">
+      <c r="F6" s="28">
         <v>0.22988505747126436</v>
       </c>
       <c r="G6">
         <v>3</v>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="28">
         <v>0.034482758620689655</v>
       </c>
       <c r="I6">
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D7">
         <v>110</v>
@@ -3477,13 +3659,13 @@
       <c r="E7">
         <v>27</v>
       </c>
-      <c r="F7" s="27">
+      <c r="F7" s="28">
         <v>0.24545454545454545</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="28">
         <v>0.01818181818181818</v>
       </c>
       <c r="I7">
@@ -3494,8 +3676,8 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
-        <v>164</v>
+      <c r="A9" s="17" t="s">
+        <v>165</v>
       </c>
       <c r="I9">
         <v>9</v>
@@ -3507,6 +3689,6 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>